<commit_message>
Quests 1.2 step 1: cleaned world riddle list (258 riddles, one-word answers with aliases), boss notes for all ten boss pairs in the monster sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/RPG_0.1.xlsx
+++ b/docs/RPG_0.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sonstiges\3D RPG\game\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC1E51E2-8CF9-4C2E-8C71-4616DD52C833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A84110-B90B-44D4-85F2-33B9373C8591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{4BE2A854-3C52-4E67-A093-93255C02F786}"/>
+    <workbookView xWindow="9345" yWindow="3465" windowWidth="28800" windowHeight="11235" xr2:uid="{4BE2A854-3C52-4E67-A093-93255C02F786}"/>
   </bookViews>
   <sheets>
     <sheet name="Monster" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="161">
   <si>
     <t>False</t>
   </si>
@@ -126,9 +126,6 @@
   </si>
   <si>
     <t>Werewolf</t>
-  </si>
-  <si>
-    <t>both</t>
   </si>
   <si>
     <t>Poison</t>
@@ -647,10 +644,6 @@
   </cellStyles>
   <dxfs count="10">
     <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -661,6 +654,10 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -725,21 +722,21 @@
     <tableColumn id="39" xr3:uid="{FE9BCC63-A58F-4EE4-AEF0-714F5229CD56}" name="entity 8l: _x000a_regeneration_per_turn_in_percent_of total_life"/>
     <tableColumn id="40" xr3:uid="{20EFEFED-5BC7-4680-8D94-F0FFDF66C696}" name="entity 8m: _x000a_steal_mana_on_hit_in_percent_of_characters_max_mana"/>
     <tableColumn id="41" xr3:uid="{6B83D3CE-7E9F-4FEC-A9B7-E09FF7C7DABE}" name="entity 8n: _x000a_increases_magical_age_by_1_year_on_hit"/>
-    <tableColumn id="10" xr3:uid="{657AB867-1E43-41EC-95BE-4DF86DC71643}" name="entity 9:_x000a_outside_spawner_hut_xp" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{657AB867-1E43-41EC-95BE-4DF86DC71643}" name="entity 9:_x000a_outside_spawner_hut_xp" dataDxfId="4"/>
     <tableColumn id="11" xr3:uid="{C864C4B0-6F86-4266-84B7-0009F0740F0B}" name="entity 10:_x000a_res_magic"/>
     <tableColumn id="12" xr3:uid="{4DE80521-738A-490D-8660-B2E4BE035E51}" name="entity 11:_x000a_res_fire"/>
     <tableColumn id="13" xr3:uid="{FEFD4387-19A1-41A1-9279-3622879EEEF7}" name="entity 12:_x000a_res_physical"/>
     <tableColumn id="15" xr3:uid="{9D486DD9-3A76-4B9D-A48E-45B8AC5A9204}" name="entity 13:_x000a_res_cold"/>
     <tableColumn id="16" xr3:uid="{674684F8-3D91-4BFB-A915-BAFCD2C82B25}" name="entity 14:_x000a_res_poison"/>
     <tableColumn id="18" xr3:uid="{4F25CA0D-398A-4ADE-B1B4-5F0BB7C038DA}" name="entity 15:_x000a_exp_old (not used anymore)"/>
-    <tableColumn id="27" xr3:uid="{BB0197D4-3C5C-4D64-BB3F-0966359DE0DF}" name="entity 16:_x000a_gold" dataDxfId="4"/>
+    <tableColumn id="27" xr3:uid="{BB0197D4-3C5C-4D64-BB3F-0966359DE0DF}" name="entity 16:_x000a_gold" dataDxfId="3"/>
     <tableColumn id="25" xr3:uid="{ED29C8D4-1AB4-48DC-AD5F-5B5BCA75AC90}" name="entity 17:_x000a_treasure_level_old (not used anymore)"/>
-    <tableColumn id="6" xr3:uid="{306F37DE-3F0E-4874-9CA6-CA8E4537DAC0}" name="entity 18:_x000a_icon_height" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{306F37DE-3F0E-4874-9CA6-CA8E4537DAC0}" name="entity 18:_x000a_icon_height" dataDxfId="2"/>
     <tableColumn id="7" xr3:uid="{06CC750E-0BC9-4044-ADAB-702E10B69198}" name="entity 19:_x000a_terrain"/>
     <tableColumn id="14" xr3:uid="{10A0D880-46D4-4EF1-9E97-94B8F7FF7F8A}" name="entity 20:_x000a_undead"/>
     <tableColumn id="17" xr3:uid="{5C125C46-427D-41B4-A8E2-C627B813F7BF}" name="entity 21:_x000a_final_boss"/>
     <tableColumn id="19" xr3:uid="{0A20AB78-3403-450A-92F0-E11B2C907395}" name="entity 22: group"/>
-    <tableColumn id="9" xr3:uid="{4D1BFE81-E36F-433A-9F94-15DAEEA44F00}" name="entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)" dataDxfId="2">
+    <tableColumn id="9" xr3:uid="{4D1BFE81-E36F-433A-9F94-15DAEEA44F00}" name="entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)" dataDxfId="1">
       <calculatedColumnFormula>(_csv247[[#This Row],[entity 1:
 health]]*_csv247[[#This Row],[entity 2:
 armor]]+_csv247[[#This Row],[entity 1:
@@ -758,7 +755,7 @@
 regeneration_per_turn_in_percent_of total_life]]*100000+_csv247[[#This Row],[entity 8m: 
 steal_mana_on_hit_in_percent_of_characters_max_mana]]*50000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{8A88862A-3CB6-4053-9301-EB3CFDFFA903}" name="entity 24: treasure_level_new" dataDxfId="1"/>
+    <tableColumn id="20" xr3:uid="{8A88862A-3CB6-4053-9301-EB3CFDFFA903}" name="entity 24: treasure_level_new" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1092,124 +1089,124 @@
   <sheetData>
     <row r="1" spans="1:40" s="3" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="W1" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="X1" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="Y1" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="AA1" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="AB1" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="AC1" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="AD1" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="AE1" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="AF1" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="AG1" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="AH1" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="AI1" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AJ1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AK1" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="W1" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="Y1" s="9" t="s">
+      <c r="AL1" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="AM1" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="Z1" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA1" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="AB1" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="AC1" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="AD1" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="AE1" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="AF1" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="AG1" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="AH1" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="AI1" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="AJ1" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="AK1" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="AL1" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="AM1" s="8" t="s">
-        <v>158</v>
-      </c>
       <c r="AN1" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.25">
@@ -1217,7 +1214,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C2">
         <v>15</v>
@@ -1241,7 +1238,7 @@
         <v>6</v>
       </c>
       <c r="J2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y2" s="10" t="s">
         <v>2</v>
@@ -1280,7 +1277,7 @@
         <v>0</v>
       </c>
       <c r="AL2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM2" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -1311,7 +1308,7 @@
         <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1335,7 +1332,7 @@
         <v>3</v>
       </c>
       <c r="J3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y3" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -1375,7 +1372,7 @@
         <v>0</v>
       </c>
       <c r="AL3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM3" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -1406,7 +1403,7 @@
         <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C4">
         <v>5</v>
@@ -1430,7 +1427,7 @@
         <v>3</v>
       </c>
       <c r="L4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y4" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -1470,7 +1467,7 @@
         <v>0</v>
       </c>
       <c r="AL4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM4" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -1501,7 +1498,7 @@
         <v>78</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C5">
         <v>25</v>
@@ -1525,7 +1522,7 @@
         <v>6</v>
       </c>
       <c r="K5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y5" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -1565,7 +1562,7 @@
         <v>0</v>
       </c>
       <c r="AL5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AM5" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -1596,7 +1593,7 @@
         <v>64</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C6">
         <v>20</v>
@@ -1620,7 +1617,7 @@
         <v>3</v>
       </c>
       <c r="Y6" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z6" s="2">
         <v>0.17</v>
@@ -1656,7 +1653,7 @@
         <v>18</v>
       </c>
       <c r="AL6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AM6" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -1687,7 +1684,7 @@
         <v>62</v>
       </c>
       <c r="B7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C7">
         <v>10</v>
@@ -1711,7 +1708,7 @@
         <v>6</v>
       </c>
       <c r="O7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y7" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -1751,7 +1748,7 @@
         <v>0</v>
       </c>
       <c r="AL7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM7" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -1782,7 +1779,7 @@
         <v>80</v>
       </c>
       <c r="B8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C8">
         <v>35</v>
@@ -1806,10 +1803,10 @@
         <v>3</v>
       </c>
       <c r="P8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z8" s="2">
         <v>0.25</v>
@@ -1845,7 +1842,7 @@
         <v>18</v>
       </c>
       <c r="AL8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AM8" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -1876,7 +1873,7 @@
         <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C9">
         <v>25</v>
@@ -1900,7 +1897,7 @@
         <v>3</v>
       </c>
       <c r="J9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y9" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -1940,7 +1937,7 @@
         <v>0</v>
       </c>
       <c r="AL9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM9" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -1971,7 +1968,7 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C10">
         <v>40</v>
@@ -1995,10 +1992,10 @@
         <v>16</v>
       </c>
       <c r="K10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z10" s="2">
         <v>0.2</v>
@@ -2034,7 +2031,7 @@
         <v>0</v>
       </c>
       <c r="AL10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AM10" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -2065,7 +2062,7 @@
         <v>46</v>
       </c>
       <c r="B11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C11">
         <v>40</v>
@@ -2122,7 +2119,7 @@
         <v>0</v>
       </c>
       <c r="AL11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM11" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -2153,7 +2150,7 @@
         <v>68</v>
       </c>
       <c r="B12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C12">
         <v>15</v>
@@ -2177,7 +2174,7 @@
         <v>6</v>
       </c>
       <c r="M12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y12" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -2217,7 +2214,7 @@
         <v>0</v>
       </c>
       <c r="AL12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM12" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -2248,7 +2245,7 @@
         <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C13">
         <v>50</v>
@@ -2269,13 +2266,13 @@
         <v>12</v>
       </c>
       <c r="I13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z13" s="2">
         <v>0.1</v>
@@ -2311,7 +2308,7 @@
         <v>0</v>
       </c>
       <c r="AL13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM13" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -2342,7 +2339,7 @@
         <v>56</v>
       </c>
       <c r="B14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C14">
         <v>20</v>
@@ -2366,7 +2363,7 @@
         <v>3</v>
       </c>
       <c r="O14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z14" s="2">
         <v>0.5</v>
@@ -2402,7 +2399,7 @@
         <v>0</v>
       </c>
       <c r="AL14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM14" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -2433,7 +2430,7 @@
         <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C15">
         <v>40</v>
@@ -2457,7 +2454,7 @@
         <v>3</v>
       </c>
       <c r="M15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y15" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -2497,7 +2494,7 @@
         <v>0</v>
       </c>
       <c r="AL15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM15" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -2528,7 +2525,7 @@
         <v>52</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C16">
         <v>40</v>
@@ -2589,7 +2586,7 @@
         <v>0</v>
       </c>
       <c r="AL16" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM16" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -2620,7 +2617,7 @@
         <v>77</v>
       </c>
       <c r="B17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C17">
         <v>50</v>
@@ -2644,13 +2641,13 @@
         <v>6</v>
       </c>
       <c r="J17" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="M17" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y17" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z17" s="2">
         <v>0.5</v>
@@ -2686,7 +2683,7 @@
         <v>0</v>
       </c>
       <c r="AL17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM17" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -2717,7 +2714,7 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C18">
         <v>70</v>
@@ -2741,10 +2738,10 @@
         <v>14</v>
       </c>
       <c r="J18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z18" s="2">
         <v>0.33</v>
@@ -2780,7 +2777,7 @@
         <v>0</v>
       </c>
       <c r="AL18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM18" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -2811,7 +2808,7 @@
         <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C19">
         <v>30</v>
@@ -2835,7 +2832,7 @@
         <v>3</v>
       </c>
       <c r="L19" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y19" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -2875,7 +2872,7 @@
         <v>0</v>
       </c>
       <c r="AL19" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM19" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -2906,7 +2903,7 @@
         <v>40</v>
       </c>
       <c r="B20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C20">
         <v>50</v>
@@ -2930,7 +2927,7 @@
         <v>3</v>
       </c>
       <c r="L20" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y20" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -2970,7 +2967,7 @@
         <v>0</v>
       </c>
       <c r="AL20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM20" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -3001,7 +2998,7 @@
         <v>51</v>
       </c>
       <c r="B21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C21">
         <v>60</v>
@@ -3025,7 +3022,7 @@
         <v>3</v>
       </c>
       <c r="Q21" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y21" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -3065,7 +3062,7 @@
         <v>0</v>
       </c>
       <c r="AL21" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM21" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -3096,7 +3093,7 @@
         <v>58</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C22">
         <v>100</v>
@@ -3117,13 +3114,13 @@
         <v>12</v>
       </c>
       <c r="I22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L22" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y22" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z22" s="2">
         <v>0.4</v>
@@ -3159,7 +3156,7 @@
         <v>0</v>
       </c>
       <c r="AL22" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM22" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -3190,7 +3187,7 @@
         <v>49</v>
       </c>
       <c r="B23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C23">
         <v>45</v>
@@ -3251,7 +3248,7 @@
         <v>0</v>
       </c>
       <c r="AL23" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM23" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -3282,7 +3279,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C24">
         <v>75</v>
@@ -3306,10 +3303,10 @@
         <v>3</v>
       </c>
       <c r="O24" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y24" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z24" s="2">
         <v>0</v>
@@ -3345,7 +3342,7 @@
         <v>0</v>
       </c>
       <c r="AL24" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM24" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -3376,7 +3373,7 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C25">
         <v>75</v>
@@ -3400,7 +3397,7 @@
         <v>3</v>
       </c>
       <c r="Q25" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z25" s="2">
         <v>0.2</v>
@@ -3436,7 +3433,7 @@
         <v>0</v>
       </c>
       <c r="AL25" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM25" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -3467,7 +3464,7 @@
         <v>63</v>
       </c>
       <c r="B26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C26">
         <v>50</v>
@@ -3491,7 +3488,7 @@
         <v>3</v>
       </c>
       <c r="L26" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y26" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -3531,7 +3528,7 @@
         <v>0</v>
       </c>
       <c r="AL26" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM26" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -3562,7 +3559,7 @@
         <v>18</v>
       </c>
       <c r="B27" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C27">
         <v>70</v>
@@ -3586,7 +3583,7 @@
         <v>3</v>
       </c>
       <c r="Y27" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z27" s="2">
         <v>0.17</v>
@@ -3622,7 +3619,7 @@
         <v>0</v>
       </c>
       <c r="AL27" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM27" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -3653,7 +3650,7 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C28">
         <v>50</v>
@@ -3677,7 +3674,7 @@
         <v>3</v>
       </c>
       <c r="N28" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z28" s="2">
         <v>0.5</v>
@@ -3713,7 +3710,7 @@
         <v>0</v>
       </c>
       <c r="AL28" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM28" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -3744,7 +3741,7 @@
         <v>55</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C29">
         <v>50</v>
@@ -3768,7 +3765,7 @@
         <v>6</v>
       </c>
       <c r="X29" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z29" s="2">
         <v>0.2</v>
@@ -3804,7 +3801,7 @@
         <v>0</v>
       </c>
       <c r="AL29" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AM29" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -3835,7 +3832,7 @@
         <v>57</v>
       </c>
       <c r="B30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C30">
         <v>40</v>
@@ -3859,7 +3856,7 @@
         <v>3</v>
       </c>
       <c r="Y30" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z30" s="2">
         <v>0</v>
@@ -3895,7 +3892,7 @@
         <v>0</v>
       </c>
       <c r="AL30" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM30" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -3926,7 +3923,7 @@
         <v>5</v>
       </c>
       <c r="B31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C31">
         <v>60</v>
@@ -3987,7 +3984,7 @@
         <v>0</v>
       </c>
       <c r="AL31" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM31" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -4018,7 +4015,7 @@
         <v>9</v>
       </c>
       <c r="B32" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C32">
         <v>100</v>
@@ -4042,10 +4039,10 @@
         <v>6</v>
       </c>
       <c r="J32" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K32" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z32" s="2">
         <v>7.0000000000000007E-2</v>
@@ -4081,7 +4078,7 @@
         <v>0</v>
       </c>
       <c r="AL32" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM32" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -4112,7 +4109,7 @@
         <v>7</v>
       </c>
       <c r="B33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C33">
         <v>40</v>
@@ -4169,7 +4166,7 @@
         <v>0</v>
       </c>
       <c r="AL33" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM33" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -4200,7 +4197,7 @@
         <v>66</v>
       </c>
       <c r="B34" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C34">
         <v>100</v>
@@ -4224,7 +4221,7 @@
         <v>16</v>
       </c>
       <c r="J34" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z34" s="2">
         <v>0</v>
@@ -4260,7 +4257,7 @@
         <v>0</v>
       </c>
       <c r="AL34" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM34" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -4291,7 +4288,7 @@
         <v>91</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C35">
         <v>250</v>
@@ -4348,10 +4345,10 @@
         <v>0</v>
       </c>
       <c r="AK35" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AL35" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM35" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -4382,7 +4379,7 @@
         <v>20</v>
       </c>
       <c r="B36" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C36">
         <v>125</v>
@@ -4439,7 +4436,7 @@
         <v>0</v>
       </c>
       <c r="AL36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM36" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -4470,7 +4467,7 @@
         <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C37">
         <v>100</v>
@@ -4494,7 +4491,7 @@
         <v>3</v>
       </c>
       <c r="Q37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y37" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -4534,7 +4531,7 @@
         <v>0</v>
       </c>
       <c r="AL37" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM37" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -4565,7 +4562,7 @@
         <v>28</v>
       </c>
       <c r="B38" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C38">
         <v>100</v>
@@ -4589,7 +4586,7 @@
         <v>6</v>
       </c>
       <c r="X38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z38" s="2">
         <v>0.15</v>
@@ -4625,7 +4622,7 @@
         <v>18</v>
       </c>
       <c r="AL38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AM38" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -4656,7 +4653,7 @@
         <v>65</v>
       </c>
       <c r="B39" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C39">
         <v>75</v>
@@ -4713,7 +4710,7 @@
         <v>0</v>
       </c>
       <c r="AL39" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM39" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -4744,7 +4741,7 @@
         <v>1</v>
       </c>
       <c r="B40" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C40">
         <v>100</v>
@@ -4768,7 +4765,7 @@
         <v>3</v>
       </c>
       <c r="J40" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y40" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -4808,7 +4805,7 @@
         <v>0</v>
       </c>
       <c r="AL40" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM40" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -4839,7 +4836,7 @@
         <v>71</v>
       </c>
       <c r="B41" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C41">
         <v>150</v>
@@ -4863,7 +4860,7 @@
         <v>3</v>
       </c>
       <c r="Y41" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z41" s="2">
         <v>0.9</v>
@@ -4899,7 +4896,7 @@
         <v>0</v>
       </c>
       <c r="AL41" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AM41" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -4930,7 +4927,7 @@
         <v>26</v>
       </c>
       <c r="B42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C42">
         <v>75</v>
@@ -4954,7 +4951,7 @@
         <v>14</v>
       </c>
       <c r="Y42" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z42" s="2">
         <v>0.27</v>
@@ -4990,7 +4987,7 @@
         <v>0</v>
       </c>
       <c r="AL42" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM42" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -5021,7 +5018,7 @@
         <v>25</v>
       </c>
       <c r="B43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C43">
         <v>150</v>
@@ -5045,10 +5042,10 @@
         <v>14</v>
       </c>
       <c r="J43" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y43" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z43" s="2">
         <v>0.05</v>
@@ -5084,7 +5081,7 @@
         <v>0</v>
       </c>
       <c r="AL43" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM43" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -5115,7 +5112,7 @@
         <v>24</v>
       </c>
       <c r="B44" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C44">
         <v>100</v>
@@ -5139,7 +5136,7 @@
         <v>3</v>
       </c>
       <c r="J44" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y44" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -5179,7 +5176,7 @@
         <v>0</v>
       </c>
       <c r="AL44" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM44" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -5210,7 +5207,7 @@
         <v>72</v>
       </c>
       <c r="B45" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C45">
         <v>125</v>
@@ -5274,7 +5271,7 @@
         <v>0</v>
       </c>
       <c r="AL45" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM45" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -5305,7 +5302,7 @@
         <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C46">
         <v>50</v>
@@ -5365,7 +5362,7 @@
         <v>0</v>
       </c>
       <c r="AL46" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM46" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -5396,7 +5393,7 @@
         <v>16</v>
       </c>
       <c r="B47" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C47">
         <v>100</v>
@@ -5420,7 +5417,7 @@
         <v>3</v>
       </c>
       <c r="P47" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y47" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -5460,7 +5457,7 @@
         <v>0</v>
       </c>
       <c r="AL47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM47" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -5491,7 +5488,7 @@
         <v>27</v>
       </c>
       <c r="B48" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C48">
         <v>125</v>
@@ -5515,10 +5512,10 @@
         <v>3</v>
       </c>
       <c r="T48" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y48" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z48" s="2">
         <v>0.1</v>
@@ -5554,7 +5551,7 @@
         <v>0</v>
       </c>
       <c r="AL48" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM48" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -5585,7 +5582,7 @@
         <v>60</v>
       </c>
       <c r="B49" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C49">
         <v>150</v>
@@ -5609,7 +5606,7 @@
         <v>6</v>
       </c>
       <c r="J49" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z49" s="2">
         <v>0.1</v>
@@ -5645,7 +5642,7 @@
         <v>18</v>
       </c>
       <c r="AL49" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AM49" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -5676,7 +5673,7 @@
         <v>2</v>
       </c>
       <c r="B50" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C50">
         <v>175</v>
@@ -5700,7 +5697,7 @@
         <v>3</v>
       </c>
       <c r="J50" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y50" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -5740,7 +5737,7 @@
         <v>0</v>
       </c>
       <c r="AL50" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM50" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -5771,7 +5768,7 @@
         <v>14</v>
       </c>
       <c r="B51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C51">
         <v>125</v>
@@ -5795,7 +5792,7 @@
         <v>3</v>
       </c>
       <c r="O51" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z51" s="2">
         <v>0.1</v>
@@ -5831,7 +5828,7 @@
         <v>0</v>
       </c>
       <c r="AL51" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM51" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -5862,7 +5859,7 @@
         <v>23</v>
       </c>
       <c r="B52" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C52">
         <v>100</v>
@@ -5886,7 +5883,7 @@
         <v>6</v>
       </c>
       <c r="O52" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z52" s="2">
         <v>0.9</v>
@@ -5922,7 +5919,7 @@
         <v>0</v>
       </c>
       <c r="AL52" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM52" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -5953,7 +5950,7 @@
         <v>44</v>
       </c>
       <c r="B53" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C53">
         <v>150</v>
@@ -5977,7 +5974,7 @@
         <v>14</v>
       </c>
       <c r="J53" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y53" s="10">
         <f>_csv247[[#This Row],[entity 23: XP_new (While entity 24 give a rough idea of where place the monsters, the XP is the fine tuning. start with the lowest XP and use higher XP monsters, the further the heroes are venturing out)]]*13</f>
@@ -6017,7 +6014,7 @@
         <v>0</v>
       </c>
       <c r="AL53" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM53" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -6048,7 +6045,7 @@
         <v>67</v>
       </c>
       <c r="B54" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C54">
         <v>100</v>
@@ -6105,7 +6102,7 @@
         <v>0</v>
       </c>
       <c r="AL54" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM54" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -6136,7 +6133,7 @@
         <v>59</v>
       </c>
       <c r="B55" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C55">
         <v>200</v>
@@ -6193,7 +6190,7 @@
         <v>0</v>
       </c>
       <c r="AL55" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM55" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -6224,7 +6221,7 @@
         <v>38</v>
       </c>
       <c r="B56" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C56">
         <v>200</v>
@@ -6248,7 +6245,7 @@
         <v>6</v>
       </c>
       <c r="S56" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z56" s="2">
         <v>0.5</v>
@@ -6284,7 +6281,7 @@
         <v>18</v>
       </c>
       <c r="AL56" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AM56" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -6315,7 +6312,7 @@
         <v>47</v>
       </c>
       <c r="B57" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C57">
         <v>250</v>
@@ -6339,7 +6336,7 @@
         <v>3</v>
       </c>
       <c r="P57" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z57" s="2">
         <v>0.6</v>
@@ -6375,7 +6372,7 @@
         <v>0</v>
       </c>
       <c r="AL57" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AM57" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -6406,7 +6403,7 @@
         <v>15</v>
       </c>
       <c r="B58" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C58">
         <v>300</v>
@@ -6427,10 +6424,10 @@
         <v>200</v>
       </c>
       <c r="I58" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L58" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z58" s="2">
         <v>0.1</v>
@@ -6466,7 +6463,7 @@
         <v>0</v>
       </c>
       <c r="AL58" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM58" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -6497,7 +6494,7 @@
         <v>34</v>
       </c>
       <c r="B59" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C59">
         <v>250</v>
@@ -6554,7 +6551,7 @@
         <v>0</v>
       </c>
       <c r="AL59" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM59" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -6585,7 +6582,7 @@
         <v>54</v>
       </c>
       <c r="B60" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C60">
         <v>175</v>
@@ -6609,10 +6606,10 @@
         <v>3</v>
       </c>
       <c r="J60" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y60" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z60" s="2">
         <v>0.5</v>
@@ -6648,7 +6645,7 @@
         <v>0</v>
       </c>
       <c r="AL60" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM60" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -6679,7 +6676,7 @@
         <v>19</v>
       </c>
       <c r="B61" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C61">
         <v>500</v>
@@ -6703,7 +6700,7 @@
         <v>3</v>
       </c>
       <c r="Y61" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z61" s="2">
         <v>0.27</v>
@@ -6739,7 +6736,7 @@
         <v>0</v>
       </c>
       <c r="AL61" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM61" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -6770,7 +6767,7 @@
         <v>81</v>
       </c>
       <c r="B62" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C62">
         <v>300</v>
@@ -6794,10 +6791,10 @@
         <v>3</v>
       </c>
       <c r="J62" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="N62" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z62" s="2">
         <v>0.2</v>
@@ -6832,8 +6829,13 @@
       <c r="AJ62" t="s">
         <v>0</v>
       </c>
+      <c r="AK62" t="inlineStr">
+        <is>
+          <t>Boss for ID10</t>
+        </is>
+      </c>
       <c r="AL62" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM62" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -6864,7 +6866,7 @@
         <v>41</v>
       </c>
       <c r="B63" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C63">
         <v>333</v>
@@ -6888,10 +6890,10 @@
         <v>3</v>
       </c>
       <c r="T63" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y63" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z63" s="2">
         <v>0.8</v>
@@ -6927,7 +6929,7 @@
         <v>0</v>
       </c>
       <c r="AL63" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM63" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -6958,7 +6960,7 @@
         <v>84</v>
       </c>
       <c r="B64" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C64">
         <v>200</v>
@@ -6982,7 +6984,7 @@
         <v>6</v>
       </c>
       <c r="O64" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z64" s="2">
         <v>0.9</v>
@@ -7017,8 +7019,13 @@
       <c r="AJ64" t="s">
         <v>0</v>
       </c>
+      <c r="AK64" t="inlineStr">
+        <is>
+          <t>Boss for ID23</t>
+        </is>
+      </c>
       <c r="AL64" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM64" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -7049,7 +7056,7 @@
         <v>35</v>
       </c>
       <c r="B65" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C65">
         <v>200</v>
@@ -7073,7 +7080,7 @@
         <v>6</v>
       </c>
       <c r="J65" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z65" s="2">
         <v>0.27</v>
@@ -7109,7 +7116,7 @@
         <v>0</v>
       </c>
       <c r="AL65" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AM65" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -7164,7 +7171,7 @@
         <v>6</v>
       </c>
       <c r="J66" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z66" s="2">
         <v>1</v>
@@ -7200,7 +7207,7 @@
         <v>0</v>
       </c>
       <c r="AL66" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM66" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -7231,7 +7238,7 @@
         <v>70</v>
       </c>
       <c r="B67" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C67">
         <v>300</v>
@@ -7255,10 +7262,10 @@
         <v>3</v>
       </c>
       <c r="L67" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y67" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z67" s="2">
         <v>0.05</v>
@@ -7294,7 +7301,7 @@
         <v>0</v>
       </c>
       <c r="AL67" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM67" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -7349,10 +7356,10 @@
         <v>14</v>
       </c>
       <c r="J68" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K68" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z68" s="2">
         <v>0.1</v>
@@ -7388,7 +7395,7 @@
         <v>0</v>
       </c>
       <c r="AL68" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AM68" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -7443,7 +7450,7 @@
         <v>3</v>
       </c>
       <c r="P69" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z69" s="2">
         <v>0.6</v>
@@ -7479,10 +7486,10 @@
         <v>0</v>
       </c>
       <c r="AK69" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="AL69" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AM69" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -7513,7 +7520,7 @@
         <v>86</v>
       </c>
       <c r="B70" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C70">
         <v>500</v>
@@ -7537,10 +7544,10 @@
         <v>6</v>
       </c>
       <c r="J70" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K70" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z70" s="2">
         <v>0.5</v>
@@ -7575,8 +7582,13 @@
       <c r="AJ70" t="s">
         <v>0</v>
       </c>
+      <c r="AK70" t="inlineStr">
+        <is>
+          <t>Boss for ID59</t>
+        </is>
+      </c>
       <c r="AL70" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM70" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -7607,7 +7619,7 @@
         <v>13</v>
       </c>
       <c r="B71" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C71">
         <v>500</v>
@@ -7631,10 +7643,10 @@
         <v>3</v>
       </c>
       <c r="O71" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y71" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z71" s="2">
         <v>0.3</v>
@@ -7670,7 +7682,7 @@
         <v>0</v>
       </c>
       <c r="AL71" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM71" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -7701,7 +7713,7 @@
         <v>17</v>
       </c>
       <c r="B72" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C72">
         <v>500</v>
@@ -7725,10 +7737,10 @@
         <v>3</v>
       </c>
       <c r="T72" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y72" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z72" s="2">
         <v>0</v>
@@ -7764,7 +7776,7 @@
         <v>0</v>
       </c>
       <c r="AL72" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM72" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -7795,7 +7807,7 @@
         <v>3</v>
       </c>
       <c r="B73" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C73">
         <v>375</v>
@@ -7819,13 +7831,13 @@
         <v>3</v>
       </c>
       <c r="J73" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Q73" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y73" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z73" s="2">
         <v>0.5</v>
@@ -7861,7 +7873,7 @@
         <v>0</v>
       </c>
       <c r="AL73" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM73" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -7892,7 +7904,7 @@
         <v>21</v>
       </c>
       <c r="B74" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C74">
         <v>400</v>
@@ -7913,16 +7925,16 @@
         <v>100</v>
       </c>
       <c r="I74" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K74" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L74" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y74" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z74" s="2">
         <v>0.2</v>
@@ -7952,13 +7964,13 @@
         <v>3.5</v>
       </c>
       <c r="AI74" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="AJ74" t="s">
         <v>0</v>
       </c>
       <c r="AL74" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM74" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -8019,7 +8031,7 @@
         <v>0.2</v>
       </c>
       <c r="Y75" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z75" s="2">
         <v>0.1</v>
@@ -8055,7 +8067,7 @@
         <v>18</v>
       </c>
       <c r="AL75" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AM75" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -8110,10 +8122,10 @@
         <v>3</v>
       </c>
       <c r="P76" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y76" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z76" s="2">
         <v>0.2</v>
@@ -8149,7 +8161,7 @@
         <v>0</v>
       </c>
       <c r="AL76" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM76" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -8180,7 +8192,7 @@
         <v>22</v>
       </c>
       <c r="B77" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C77">
         <v>400</v>
@@ -8204,7 +8216,7 @@
         <v>6</v>
       </c>
       <c r="J77" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z77" s="2">
         <v>0.33</v>
@@ -8240,7 +8252,7 @@
         <v>0</v>
       </c>
       <c r="AL77" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AM77" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -8295,7 +8307,7 @@
         <v>3</v>
       </c>
       <c r="Y78" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z78" s="2">
         <v>0.2</v>
@@ -8331,7 +8343,7 @@
         <v>0</v>
       </c>
       <c r="AL78" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM78" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -8386,7 +8398,7 @@
         <v>3</v>
       </c>
       <c r="N79" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z79" s="2">
         <v>0.9</v>
@@ -8422,7 +8434,7 @@
         <v>0</v>
       </c>
       <c r="AL79" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM79" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -8477,7 +8489,7 @@
         <v>3</v>
       </c>
       <c r="O80" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z80" s="2">
         <v>0.8</v>
@@ -8512,8 +8524,13 @@
       <c r="AJ80" t="s">
         <v>0</v>
       </c>
+      <c r="AK80" t="inlineStr">
+        <is>
+          <t>Boss for ID13</t>
+        </is>
+      </c>
       <c r="AL80" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AM80" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -8568,7 +8585,7 @@
         <v>16</v>
       </c>
       <c r="J81" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z81" s="2">
         <v>0.25</v>
@@ -8604,7 +8621,7 @@
         <v>0</v>
       </c>
       <c r="AL81" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM81" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -8691,11 +8708,13 @@
       <c r="AJ82" t="s">
         <v>0</v>
       </c>
-      <c r="AK82" t="s">
-        <v>123</v>
+      <c r="AK82" t="inlineStr">
+        <is>
+          <t>Boss for ID36</t>
+        </is>
       </c>
       <c r="AL82" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AM82" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -8789,10 +8808,10 @@
         <v>18</v>
       </c>
       <c r="AK83" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="AL83" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AM83" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -8847,13 +8866,13 @@
         <v>6</v>
       </c>
       <c r="J84" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="R84" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="S84" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z84" s="2">
         <v>0.8</v>
@@ -8889,7 +8908,7 @@
         <v>0</v>
       </c>
       <c r="AL84" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AM84" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -8944,7 +8963,7 @@
         <v>14</v>
       </c>
       <c r="J85" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z85" s="2">
         <v>0.5</v>
@@ -8980,10 +8999,10 @@
         <v>0</v>
       </c>
       <c r="AK85" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AL85" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM85" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -9038,7 +9057,7 @@
         <v>3</v>
       </c>
       <c r="S86" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z86" s="2">
         <v>1</v>
@@ -9074,7 +9093,7 @@
         <v>0</v>
       </c>
       <c r="AL86" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM86" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -9129,10 +9148,10 @@
         <v>3</v>
       </c>
       <c r="T87" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y87" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z87" s="2">
         <v>0.2</v>
@@ -9168,7 +9187,7 @@
         <v>0</v>
       </c>
       <c r="AL87" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM87" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -9223,7 +9242,7 @@
         <v>6</v>
       </c>
       <c r="U88" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z88" s="2">
         <v>0.33</v>
@@ -9259,7 +9278,7 @@
         <v>0</v>
       </c>
       <c r="AL88" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="AM88" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -9314,10 +9333,10 @@
         <v>3</v>
       </c>
       <c r="Q89" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y89" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z89" s="2">
         <v>0.27</v>
@@ -9353,7 +9372,7 @@
         <v>0</v>
       </c>
       <c r="AL89" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM89" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -9408,10 +9427,10 @@
         <v>3</v>
       </c>
       <c r="T90" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Y90" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z90" s="2">
         <v>0.15</v>
@@ -9447,7 +9466,7 @@
         <v>0</v>
       </c>
       <c r="AL90" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM90" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -9535,10 +9554,10 @@
         <v>0</v>
       </c>
       <c r="AK91" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL91" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM91" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -9593,7 +9612,7 @@
         <v>3</v>
       </c>
       <c r="L92" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Z92" s="2">
         <v>0.1</v>
@@ -9629,7 +9648,7 @@
         <v>0</v>
       </c>
       <c r="AL92" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AM92" s="6">
         <f>(_csv247[[#This Row],[entity 1:
@@ -9692,21 +9711,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B1" t="s">
         <v>152</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>153</v>
-      </c>
-      <c r="C1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" t="s">
         <v>150</v>
-      </c>
-      <c r="B2" t="s">
-        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -9728,7 +9747,7 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>